<commit_message>
Add sample rows to data/shala-events.xlsx for preview
Two clearly-labeled (Sample) rows — one current, one future — using the
existing shala logo as a placeholder flyer/image, so the Shala Events
cards + flyer modal can be previewed on the live site. Replace or
delete via the admin panel once verified.
</commit_message>
<xml_diff>
--- a/data/shala-events.xlsx
+++ b/data/shala-events.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -515,6 +515,142 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Shala Winter Picnic (Sample)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Community Hall</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Westborough, MA</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>shala@sankalpmarathimandal.org</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>11:00 AM - 2:00 PM</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Sample placeholder data — replace or delete this row in the admin panel once verified.</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Sample placeholder data — replace or delete this row in the admin panel once verified. Games, snacks, and a group Marathi sing-along for all Shala families.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>assets/images/branding/shala-logo.jpg</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>assets/images/branding/shala-logo.jpg</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>future</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Shala Annual Day (Sample)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Sankalp Auditorium</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Marlborough, MA</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>shala@sankalpmarathimandal.org</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>4:00 PM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Sample placeholder data — replace or delete this row in the admin panel once verified.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Sample placeholder data — replace or delete this row in the admin panel once verified. Students showcase a year of Marathi learning with skits, songs, and recitations.</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>assets/images/branding/shala-logo.jpg</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>assets/images/branding/shala-logo.jpg</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
Admin: edit data/shala-events.xlsx via table editor
</commit_message>
<xml_diff>
--- a/data/shala-events.xlsx
+++ b/data/shala-events.xlsx
@@ -478,10 +478,10 @@
         <v>Book Distribution for new batch of 2026-2027</v>
       </c>
       <c r="L2" t="str">
-        <v>assets/images/branding/shala-logo.jpg</v>
+        <v>assets/images/shala/events/Bookdistribution.jpeg</v>
       </c>
       <c r="M2" t="str">
-        <v>assets/images/branding/shala-logo.jpg</v>
+        <v>assets/images/shala/events/Bookdistribution.jpeg</v>
       </c>
       <c r="N2" t="str">
         <v/>

</xml_diff>